<commit_message>
feat: explicitly request RUT, Full Name, DOB and Relationship in Excel KYC template and improve parser
</commit_message>
<xml_diff>
--- a/PRINCIPAL/PRODUCTOS/SEGURO DE VIDA CON AHORRO PREFERENTE/Formulario_Cliente_DPS.xlsx
+++ b/PRINCIPAL/PRODUCTOS/SEGURO DE VIDA CON AHORRO PREFERENTE/Formulario_Cliente_DPS.xlsx
@@ -640,20 +640,20 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="63" customHeight="1">
+    <row r="5" ht="95" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Detalle de Herederos (Parentesco y Composición Familiar)</t>
+          <t>Detalle de Herederos (Parentesco, RUT, Fecha de Nacimiento y Nombre Completo)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Requerido para la planificación de sucesión, cálculo de exenciones tributarias y distribución legal eficiente.</t>
+          <t>Requerido para la planificación de sucesión, cálculo de exenciones tributarias de herencia (Ley N° 16.271) y tabla actuarial de distribución.</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Escriba nombres y parentesco. Ej: María González (Cónyuge - 50%), Pedro Pérez (Hijo - 25%), Ana Pérez (Hija - 25%). NO responder solo 'Sí'.</t>
+          <t>Indique RUT, Nombre Completo, Fecha de Nacimiento (DD/MM/AAAA) y Parentesco. Ej: 9.017.656-0 Rosa Henríquez Contreras (Fecha Nac: 15/05/1958 - Cónyuge - 50%), 15.870.820-4 Ignacio González Henríquez (Fecha Nac: 20/10/1985 - Hijo - 25%), 18.234.567-1 Isidora González Henríquez (Fecha Nac: 04/12/1992 - Hija - 25%). NO responder solo 'Sí'.</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr"/>

</xml_diff>